<commit_message>
Mise à jour site Bois
</commit_message>
<xml_diff>
--- a/prix/prix.xlsx
+++ b/prix/prix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\bois\prix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E84DA782-E6E9-455D-BD8B-3B9CC28C588B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65EA6416-431E-471D-A6EC-6BB520C2710C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="19416" windowHeight="11016" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
+    <workbookView xWindow="23124" yWindow="0" windowWidth="19116" windowHeight="10884" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="474">
   <si>
     <t>path</t>
   </si>
@@ -1449,6 +1449,15 @@
   </si>
   <si>
     <t>OSB22-59x244-Sterling</t>
+  </si>
+  <si>
+    <t>11201110</t>
+  </si>
+  <si>
+    <t>OSB III 15 rainuré 59x244 KRONO</t>
+  </si>
+  <si>
+    <t>OSB15-59x244-krono</t>
   </si>
 </sst>
 </file>
@@ -1532,7 +1541,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1602,6 +1611,34 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -1938,7 +1975,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{065E4AF0-A4F8-4CE3-9E23-EDCEACB756BD}">
-  <dimension ref="A1:G453"/>
+  <dimension ref="A1:G454"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="37" style="4" bestFit="1" customWidth="1"/>
@@ -1969,7 +2006,7 @@
       <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="10"/>
+      <c r="G1" s="26"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
@@ -1981,16 +2018,16 @@
       <c r="C2" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="28">
         <v>15.44</v>
       </c>
       <c r="E2" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="12">
-        <v>104.88500000000023</v>
-      </c>
-      <c r="G2" s="10"/>
+      <c r="F2" s="29">
+        <v>95.495000000000232</v>
+      </c>
+      <c r="G2" s="26"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
@@ -2002,16 +2039,16 @@
       <c r="C3" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="D3" s="11">
+      <c r="D3" s="28">
         <v>18.73</v>
       </c>
       <c r="E3" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="12">
+      <c r="F3" s="29">
         <v>0</v>
       </c>
-      <c r="G3" s="10"/>
+      <c r="G3" s="26"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
@@ -2023,16 +2060,16 @@
       <c r="C4" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="28">
         <v>8.81</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="12">
-        <v>132.01899999999907</v>
-      </c>
-      <c r="G4" s="10"/>
+      <c r="F4" s="29">
+        <v>1.4389999999990435</v>
+      </c>
+      <c r="G4" s="26"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
@@ -2044,579 +2081,579 @@
       <c r="C5" s="2" t="s">
         <v>468</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="28">
         <v>10.78</v>
       </c>
       <c r="E5" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="12">
-        <v>256.31999999999971</v>
-      </c>
-      <c r="G5" s="10"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F5" s="29">
+        <v>210.23999999999972</v>
+      </c>
+      <c r="G5" s="26"/>
+    </row>
+    <row r="6" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>307</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>465</v>
-      </c>
-      <c r="D6" s="11">
-        <v>8.01</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>461</v>
-      </c>
-      <c r="F6" s="12">
-        <v>374.22</v>
-      </c>
-      <c r="G6" s="10"/>
+        <v>473</v>
+      </c>
+      <c r="D6" s="28">
+        <v>9.91</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>471</v>
+      </c>
+      <c r="F6" s="29">
+        <v>172.8</v>
+      </c>
+      <c r="G6" s="26"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>307</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="D7" s="11">
-        <v>11.33</v>
+        <v>465</v>
+      </c>
+      <c r="D7" s="28">
+        <v>8.16</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="F7" s="12">
-        <v>287.92</v>
-      </c>
-      <c r="G7" s="10"/>
+        <v>461</v>
+      </c>
+      <c r="F7" s="29">
+        <v>613.86000000000013</v>
+      </c>
+      <c r="G7" s="26"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>307</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>79</v>
+        <v>464</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="D8" s="11">
-        <v>12.41</v>
-      </c>
-      <c r="E8" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="12">
-        <v>374.39999999999981</v>
-      </c>
-      <c r="G8" s="10"/>
+        <v>466</v>
+      </c>
+      <c r="D8" s="28">
+        <v>11.52</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>462</v>
+      </c>
+      <c r="F8" s="29">
+        <v>548.55999999999995</v>
+      </c>
+      <c r="G8" s="26"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>307</v>
       </c>
       <c r="B9" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="D9" s="28">
+        <v>12.41</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="29">
+        <v>96.479999999999819</v>
+      </c>
+      <c r="G9" s="26"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D10" s="28">
         <v>15.74</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E10" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="12">
-        <v>83.518000000000654</v>
-      </c>
-      <c r="G9" s="10"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="D10" s="11">
-        <v>14.71</v>
-      </c>
-      <c r="E10" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="12">
-        <v>30</v>
-      </c>
-      <c r="G10" s="10"/>
+      <c r="F10" s="29">
+        <v>55.158000000000648</v>
+      </c>
+      <c r="G10" s="26"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="D11" s="11">
-        <v>22.580000000000002</v>
+        <v>81</v>
+      </c>
+      <c r="D11" s="28">
+        <v>15.51</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="12">
-        <v>90</v>
-      </c>
-      <c r="G11" s="10"/>
+        <v>12</v>
+      </c>
+      <c r="F11" s="29">
+        <v>117</v>
+      </c>
+      <c r="G11" s="26"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="D12" s="11">
-        <v>44.06</v>
+        <v>82</v>
+      </c>
+      <c r="D12" s="28">
+        <v>22.580000000000002</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="F12" s="12">
-        <v>11.519999999999982</v>
-      </c>
-      <c r="G12" s="10"/>
+        <v>13</v>
+      </c>
+      <c r="F12" s="29">
+        <v>60</v>
+      </c>
+      <c r="G12" s="26"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="D13" s="11">
-        <v>91.48</v>
+        <v>83</v>
+      </c>
+      <c r="D13" s="28">
+        <v>44.06</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="12">
-        <v>0</v>
-      </c>
-      <c r="G13" s="10"/>
+        <v>14</v>
+      </c>
+      <c r="F13" s="29">
+        <v>11.519999999999982</v>
+      </c>
+      <c r="G13" s="26"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="D14" s="28">
+        <v>91.48</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="29">
+        <v>0</v>
+      </c>
+      <c r="G14" s="26"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="5"/>
+      <c r="B15" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D15" s="28">
         <v>2.31</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E15" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F15" s="29">
         <v>0</v>
       </c>
-      <c r="G14" s="10"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="D15" s="11">
-        <v>7.79</v>
-      </c>
-      <c r="E15" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="F15" s="12">
-        <v>14.900000000000224</v>
-      </c>
-      <c r="G15" s="10"/>
+      <c r="G15" s="26"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="D16" s="11">
-        <v>10.83</v>
+        <v>313</v>
+      </c>
+      <c r="D16" s="28">
+        <v>7.79</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="F16" s="12">
-        <v>32.024999999999835</v>
-      </c>
-      <c r="G16" s="10"/>
+        <v>17</v>
+      </c>
+      <c r="F16" s="29">
+        <v>5.9600000000002238</v>
+      </c>
+      <c r="G16" s="26"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>304</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="D17" s="11">
-        <v>13.94</v>
+        <v>314</v>
+      </c>
+      <c r="D17" s="28">
+        <v>8.49</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="F17" s="12">
-        <v>4.4750000000002101</v>
-      </c>
-      <c r="G17" s="10"/>
+        <v>18</v>
+      </c>
+      <c r="F17" s="29">
+        <v>68.699999999999832</v>
+      </c>
+      <c r="G17" s="26"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>304</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="D18" s="11">
-        <v>0</v>
+        <v>315</v>
+      </c>
+      <c r="D18" s="28">
+        <v>12.8</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="F18" s="12">
-        <v>0</v>
-      </c>
-      <c r="G18" s="10"/>
+        <v>19</v>
+      </c>
+      <c r="F18" s="29">
+        <v>41.070000000000206</v>
+      </c>
+      <c r="G18" s="26"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>304</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="D19" s="11">
-        <v>20.09</v>
+        <v>316</v>
+      </c>
+      <c r="D19" s="28">
+        <v>0</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="F19" s="12">
-        <v>4.9999999981578114E-3</v>
-      </c>
-      <c r="G19" s="10"/>
+        <v>20</v>
+      </c>
+      <c r="F19" s="29">
+        <v>0</v>
+      </c>
+      <c r="G19" s="26"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>304</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="D20" s="11">
-        <v>16.75</v>
+        <v>317</v>
+      </c>
+      <c r="D20" s="28">
+        <v>16.34</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="F20" s="12">
-        <v>0</v>
-      </c>
-      <c r="G20" s="10"/>
+        <v>21</v>
+      </c>
+      <c r="F20" s="29">
+        <v>45.754999999998162</v>
+      </c>
+      <c r="G20" s="26"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>304</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="D21" s="11">
-        <v>19.990000000000002</v>
+        <v>318</v>
+      </c>
+      <c r="D21" s="28">
+        <v>16.75</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="F21" s="12">
-        <v>120.08799999999336</v>
-      </c>
-      <c r="G21" s="10"/>
+        <v>22</v>
+      </c>
+      <c r="F21" s="29">
+        <v>0</v>
+      </c>
+      <c r="G21" s="26"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>304</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="D22" s="11">
-        <v>28.560000000000002</v>
+        <v>92</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="D22" s="28">
+        <v>19.990000000000002</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="F22" s="12">
-        <v>167.15000000000467</v>
-      </c>
-      <c r="G22" s="10"/>
+        <v>23</v>
+      </c>
+      <c r="F22" s="29">
+        <v>74.87299999999334</v>
+      </c>
+      <c r="G22" s="26"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>304</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>321</v>
-      </c>
-      <c r="D23" s="11">
-        <v>28.34</v>
+        <v>320</v>
+      </c>
+      <c r="D23" s="28">
+        <v>28.560000000000002</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F23" s="12">
-        <v>144.26200000000185</v>
-      </c>
-      <c r="G23" s="10"/>
+        <v>24</v>
+      </c>
+      <c r="F23" s="29">
+        <v>166.91500000000465</v>
+      </c>
+      <c r="G23" s="26"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>304</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="D24" s="11">
-        <v>54.51</v>
+        <v>94</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="D24" s="28">
+        <v>28.34</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="F24" s="12">
-        <v>-4.9999999999914557E-3</v>
-      </c>
-      <c r="G24" s="10"/>
+        <v>25</v>
+      </c>
+      <c r="F24" s="29">
+        <v>119.86200000000186</v>
+      </c>
+      <c r="G24" s="26"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>304</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="D25" s="11">
-        <v>39.340000000000003</v>
+        <v>322</v>
+      </c>
+      <c r="D25" s="28">
+        <v>54.51</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="F25" s="12">
-        <v>0</v>
-      </c>
-      <c r="G25" s="10"/>
+        <v>26</v>
+      </c>
+      <c r="F25" s="29">
+        <v>-4.9999999999914557E-3</v>
+      </c>
+      <c r="G25" s="26"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="D26" s="11">
-        <v>9.4500000000000011</v>
+        <v>323</v>
+      </c>
+      <c r="D26" s="28">
+        <v>39.340000000000003</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="F26" s="12">
-        <v>35.736999999999895</v>
-      </c>
-      <c r="G26" s="10"/>
+        <v>27</v>
+      </c>
+      <c r="F26" s="29">
+        <v>0</v>
+      </c>
+      <c r="G26" s="26"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="D27" s="11">
-        <v>10.39</v>
+        <v>324</v>
+      </c>
+      <c r="D27" s="28">
+        <v>9.4500000000000011</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="F27" s="12">
-        <v>0</v>
-      </c>
-      <c r="G27" s="10"/>
+        <v>28</v>
+      </c>
+      <c r="F27" s="29">
+        <v>35.736999999999895</v>
+      </c>
+      <c r="G27" s="26"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="D28" s="11">
-        <v>8.98</v>
+        <v>325</v>
+      </c>
+      <c r="D28" s="28">
+        <v>10.39</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="F28" s="12">
-        <v>65.337999999999596</v>
-      </c>
-      <c r="G28" s="10"/>
+        <v>29</v>
+      </c>
+      <c r="F28" s="29">
+        <v>0</v>
+      </c>
+      <c r="G28" s="26"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="D29" s="11">
-        <v>10.81</v>
+        <v>326</v>
+      </c>
+      <c r="D29" s="28">
+        <v>8.98</v>
       </c>
       <c r="E29" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="F29" s="12">
-        <v>142.54700000000011</v>
-      </c>
-      <c r="G29" s="10"/>
+        <v>30</v>
+      </c>
+      <c r="F29" s="29">
+        <v>59.387999999999607</v>
+      </c>
+      <c r="G29" s="26"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="D30" s="11">
-        <v>8.8000000000000007</v>
+        <v>327</v>
+      </c>
+      <c r="D30" s="28">
+        <v>10.81</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="F30" s="12">
-        <v>0</v>
-      </c>
-      <c r="G30" s="10"/>
+        <v>31</v>
+      </c>
+      <c r="F30" s="29">
+        <v>133.08700000000013</v>
+      </c>
+      <c r="G30" s="26"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>330</v>
-      </c>
-      <c r="D31" s="11">
-        <v>16.080000000000002</v>
+        <v>328</v>
+      </c>
+      <c r="D31" s="28">
+        <v>8.8000000000000007</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="F31" s="12">
-        <v>176.0489999999939</v>
-      </c>
-      <c r="G31" s="10"/>
+        <v>32</v>
+      </c>
+      <c r="F31" s="29">
+        <v>0</v>
+      </c>
+      <c r="G31" s="26"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="D32" s="11">
-        <v>15.71</v>
+        <v>330</v>
+      </c>
+      <c r="D32" s="28">
+        <v>16.080000000000002</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="F32" s="12">
-        <v>0</v>
-      </c>
-      <c r="G32" s="10"/>
+        <v>33</v>
+      </c>
+      <c r="F32" s="29">
+        <v>116.55199999999391</v>
+      </c>
+      <c r="G32" s="26"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>331</v>
-      </c>
-      <c r="D33" s="11">
-        <v>31.3</v>
+        <v>329</v>
+      </c>
+      <c r="D33" s="28">
+        <v>15.71</v>
       </c>
       <c r="E33" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="F33" s="12">
+        <v>34</v>
+      </c>
+      <c r="F33" s="29">
         <v>0</v>
       </c>
-      <c r="G33" s="10"/>
+      <c r="G33" s="26"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
@@ -2626,774 +2663,779 @@
         <v>104</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>332</v>
-      </c>
-      <c r="D34" s="11">
+        <v>331</v>
+      </c>
+      <c r="D34" s="28">
         <v>31.3</v>
       </c>
       <c r="E34" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="F34" s="12">
+        <v>35</v>
+      </c>
+      <c r="F34" s="29">
         <v>0</v>
       </c>
-      <c r="G34" s="10"/>
+      <c r="G34" s="26"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="D35" s="11">
-        <v>12.98</v>
+        <v>332</v>
+      </c>
+      <c r="D35" s="28">
+        <v>31.3</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="F35" s="12">
-        <v>152.56700000000018</v>
-      </c>
-      <c r="G35" s="10"/>
+        <v>36</v>
+      </c>
+      <c r="F35" s="29">
+        <v>0</v>
+      </c>
+      <c r="G35" s="26"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="D36" s="11">
-        <v>18.11</v>
+        <v>336</v>
+      </c>
+      <c r="D36" s="28">
+        <v>12.98</v>
       </c>
       <c r="E36" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="F36" s="12">
-        <v>152.87599999999372</v>
-      </c>
-      <c r="G36" s="10"/>
+        <v>37</v>
+      </c>
+      <c r="F36" s="29">
+        <v>146.60700000000017</v>
+      </c>
+      <c r="G36" s="26"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>333</v>
-      </c>
-      <c r="D37" s="11">
-        <v>18.97</v>
+        <v>335</v>
+      </c>
+      <c r="D37" s="28">
+        <v>18.11</v>
       </c>
       <c r="E37" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="F37" s="12">
-        <v>0</v>
-      </c>
-      <c r="G37" s="10"/>
+        <v>38</v>
+      </c>
+      <c r="F37" s="29">
+        <v>69.620999999993714</v>
+      </c>
+      <c r="G37" s="26"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="D38" s="11">
-        <v>24.560000000000002</v>
+        <v>333</v>
+      </c>
+      <c r="D38" s="28">
+        <v>18.97</v>
       </c>
       <c r="E38" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="F38" s="12">
+        <v>39</v>
+      </c>
+      <c r="F38" s="29">
         <v>0</v>
       </c>
-      <c r="G38" s="10"/>
+      <c r="G38" s="26"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="D39" s="11">
-        <v>56.24</v>
+        <v>339</v>
+      </c>
+      <c r="D39" s="28">
+        <v>24.560000000000002</v>
       </c>
       <c r="E39" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="F39" s="12">
+        <v>40</v>
+      </c>
+      <c r="F39" s="29">
         <v>0</v>
       </c>
-      <c r="G39" s="10"/>
+      <c r="G39" s="26"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D40" s="11">
-        <v>91.48</v>
+        <v>340</v>
+      </c>
+      <c r="D40" s="28">
+        <v>56.24</v>
       </c>
       <c r="E40" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="F40" s="12">
+        <v>41</v>
+      </c>
+      <c r="F40" s="29">
         <v>0</v>
       </c>
-      <c r="G40" s="10"/>
+      <c r="G40" s="26"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B41" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="D41" s="28">
+        <v>91.48</v>
+      </c>
+      <c r="E41" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="F41" s="29">
+        <v>0</v>
+      </c>
+      <c r="G41" s="26"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="B42" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C42" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="D41" s="11">
+      <c r="D42" s="28">
         <v>30.060000000000002</v>
       </c>
-      <c r="E41" s="19" t="s">
+      <c r="E42" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="F41" s="12">
+      <c r="F42" s="29">
         <v>87.61900000000422</v>
       </c>
-      <c r="G41" s="10"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A42" s="5"/>
-      <c r="B42" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="D42" s="11">
-        <v>34.82</v>
-      </c>
-      <c r="E42" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="F42" s="12">
-        <v>0</v>
-      </c>
-      <c r="G42" s="10"/>
+      <c r="G42" s="26"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="5"/>
       <c r="B43" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="D43" s="11">
-        <v>16.64</v>
+        <v>112</v>
+      </c>
+      <c r="D43" s="28">
+        <v>34.82</v>
       </c>
       <c r="E43" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="F43" s="12">
+        <v>44</v>
+      </c>
+      <c r="F43" s="29">
         <v>0</v>
       </c>
-      <c r="G43" s="10"/>
+      <c r="G43" s="26"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="5"/>
       <c r="B44" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="D44" s="11">
-        <v>24.72</v>
+        <v>113</v>
+      </c>
+      <c r="D44" s="28">
+        <v>16.64</v>
       </c>
       <c r="E44" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="F44" s="12">
-        <v>2.34</v>
-      </c>
-      <c r="G44" s="10"/>
+        <v>45</v>
+      </c>
+      <c r="F44" s="29">
+        <v>0</v>
+      </c>
+      <c r="G44" s="26"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="5"/>
       <c r="B45" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="D45" s="11">
-        <v>25.16</v>
+        <v>114</v>
+      </c>
+      <c r="D45" s="28">
+        <v>24.72</v>
       </c>
       <c r="E45" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="F45" s="12">
-        <v>4.3964831775156199E-14</v>
-      </c>
-      <c r="G45" s="10"/>
+        <v>46</v>
+      </c>
+      <c r="F45" s="29">
+        <v>2.34</v>
+      </c>
+      <c r="G45" s="26"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="5"/>
       <c r="B46" s="14" t="s">
-        <v>116</v>
-      </c>
-      <c r="D46" s="11">
-        <v>28.8</v>
+        <v>115</v>
+      </c>
+      <c r="D46" s="28">
+        <v>25.16</v>
       </c>
       <c r="E46" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="F46" s="12">
-        <v>0</v>
-      </c>
-      <c r="G46" s="10"/>
+        <v>47</v>
+      </c>
+      <c r="F46" s="29">
+        <v>4.3964831775156199E-14</v>
+      </c>
+      <c r="G46" s="26"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="5"/>
       <c r="B47" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="D47" s="11">
-        <v>52.6</v>
+        <v>116</v>
+      </c>
+      <c r="D47" s="28">
+        <v>28.8</v>
       </c>
       <c r="E47" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="F47" s="12">
+        <v>48</v>
+      </c>
+      <c r="F47" s="29">
         <v>0</v>
       </c>
-      <c r="G47" s="10"/>
+      <c r="G47" s="26"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="5"/>
       <c r="B48" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="D48" s="11">
-        <v>33.380000000000003</v>
+        <v>117</v>
+      </c>
+      <c r="D48" s="28">
+        <v>52.6</v>
       </c>
       <c r="E48" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="F48" s="12">
+        <v>49</v>
+      </c>
+      <c r="F48" s="29">
         <v>0</v>
       </c>
-      <c r="G48" s="10"/>
+      <c r="G48" s="26"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="5"/>
       <c r="B49" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="D49" s="11">
-        <v>40.730000000000004</v>
+        <v>118</v>
+      </c>
+      <c r="D49" s="28">
+        <v>33.380000000000003</v>
       </c>
       <c r="E49" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="F49" s="12">
+        <v>50</v>
+      </c>
+      <c r="F49" s="29">
         <v>0</v>
       </c>
-      <c r="G49" s="10"/>
+      <c r="G49" s="26"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="5"/>
       <c r="B50" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="D50" s="11">
-        <v>85.05</v>
+        <v>119</v>
+      </c>
+      <c r="D50" s="28">
+        <v>40.730000000000004</v>
       </c>
       <c r="E50" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="F50" s="12">
+        <v>51</v>
+      </c>
+      <c r="F50" s="29">
         <v>0</v>
       </c>
-      <c r="G50" s="10"/>
+      <c r="G50" s="26"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="5"/>
       <c r="B51" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="D51" s="28">
+        <v>85.05</v>
+      </c>
+      <c r="E51" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F51" s="29">
+        <v>0</v>
+      </c>
+      <c r="G51" s="26"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" s="5"/>
+      <c r="B52" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="D51" s="11">
+      <c r="D52" s="28">
         <v>97.73</v>
       </c>
-      <c r="E51" s="19" t="s">
+      <c r="E52" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="F51" s="12">
+      <c r="F52" s="29">
         <v>0</v>
       </c>
-      <c r="G51" s="10"/>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A52" s="5" t="s">
-        <v>306</v>
-      </c>
-      <c r="B52" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="D52" s="11">
-        <v>30.95</v>
-      </c>
-      <c r="E52" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="F52" s="12">
-        <v>4.6799999999999837</v>
-      </c>
-      <c r="G52" s="10"/>
+      <c r="G52" s="26"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
         <v>306</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>343</v>
-      </c>
-      <c r="D53" s="11">
-        <v>25.310000000000002</v>
+        <v>342</v>
+      </c>
+      <c r="D53" s="28">
+        <v>30.95</v>
       </c>
       <c r="E53" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="F53" s="12">
-        <v>10.921000000000276</v>
-      </c>
-      <c r="G53" s="10"/>
+        <v>54</v>
+      </c>
+      <c r="F53" s="29">
+        <v>4.6799999999999837</v>
+      </c>
+      <c r="G53" s="26"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
         <v>306</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="D54" s="11">
-        <v>26.55</v>
+        <v>343</v>
+      </c>
+      <c r="D54" s="28">
+        <v>25.310000000000002</v>
       </c>
       <c r="E54" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="F54" s="12">
-        <v>80.649999999997618</v>
-      </c>
-      <c r="G54" s="10"/>
+        <v>55</v>
+      </c>
+      <c r="F54" s="29">
+        <v>1.0000000002738929E-3</v>
+      </c>
+      <c r="G54" s="26"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
         <v>306</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>345</v>
-      </c>
-      <c r="D55" s="11">
-        <v>37.869999999999997</v>
+        <v>344</v>
+      </c>
+      <c r="D55" s="28">
+        <v>15.790000000000001</v>
       </c>
       <c r="E55" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="F55" s="12">
-        <v>-3.3010000000018076</v>
-      </c>
-      <c r="G55" s="10"/>
+        <v>56</v>
+      </c>
+      <c r="F55" s="29">
+        <v>255.1349999999976</v>
+      </c>
+      <c r="G55" s="26"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
         <v>306</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="D56" s="11">
-        <v>22.59</v>
+        <v>345</v>
+      </c>
+      <c r="D56" s="28">
+        <v>37.869999999999997</v>
       </c>
       <c r="E56" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="F56" s="12">
-        <v>134.36999999999941</v>
-      </c>
-      <c r="G56" s="10"/>
+        <v>57</v>
+      </c>
+      <c r="F56" s="29">
+        <v>-5.611000000001809</v>
+      </c>
+      <c r="G56" s="26"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
         <v>306</v>
       </c>
       <c r="B57" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="D57" s="28">
+        <v>22.59</v>
+      </c>
+      <c r="E57" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="F57" s="29">
+        <v>93.809999999999405</v>
+      </c>
+      <c r="G57" s="26"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="B58" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="C58" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="D57" s="11">
+      <c r="D58" s="28">
         <v>33.380000000000003</v>
       </c>
-      <c r="E57" s="19" t="s">
+      <c r="E58" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="F57" s="12">
-        <v>95.970000000011566</v>
-      </c>
-      <c r="G57" s="10"/>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A58" s="5"/>
-      <c r="B58" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="D58" s="11">
-        <v>71.77</v>
-      </c>
-      <c r="E58" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="F58" s="12">
-        <v>0</v>
-      </c>
-      <c r="G58" s="10"/>
+      <c r="F58" s="29">
+        <v>53.810000000011556</v>
+      </c>
+      <c r="G58" s="26"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="5"/>
       <c r="B59" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="D59" s="28">
+        <v>71.77</v>
+      </c>
+      <c r="E59" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="F59" s="29">
+        <v>0</v>
+      </c>
+      <c r="G59" s="26"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60" s="5"/>
+      <c r="B60" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="D59" s="11">
+      <c r="D60" s="28">
         <v>68.930000000000007</v>
       </c>
-      <c r="E59" s="19" t="s">
+      <c r="E60" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="F59" s="12">
+      <c r="F60" s="29">
         <v>0</v>
       </c>
-      <c r="G59" s="10"/>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A60" s="5" t="s">
-        <v>306</v>
-      </c>
-      <c r="B60" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="D60" s="11">
-        <v>47.94</v>
-      </c>
-      <c r="E60" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="F60" s="12">
-        <v>62.399999999999942</v>
-      </c>
-      <c r="G60" s="10"/>
+      <c r="G60" s="26"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>306</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C61" s="2" t="s">
         <v>350</v>
       </c>
-      <c r="D61" s="11">
-        <v>25.18</v>
+      <c r="D61" s="28">
+        <v>47.94</v>
       </c>
       <c r="E61" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="F61" s="12">
-        <v>0</v>
-      </c>
-      <c r="G61" s="10"/>
+        <v>62</v>
+      </c>
+      <c r="F61" s="29">
+        <v>57.399999999999942</v>
+      </c>
+      <c r="G61" s="26"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
         <v>306</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>351</v>
-      </c>
-      <c r="D62" s="11">
-        <v>39.07</v>
+        <v>350</v>
+      </c>
+      <c r="D62" s="28">
+        <v>34.85</v>
       </c>
       <c r="E62" s="19" t="s">
-        <v>64</v>
-      </c>
-      <c r="F62" s="12">
+        <v>63</v>
+      </c>
+      <c r="F62" s="29">
         <v>0</v>
       </c>
-      <c r="G62" s="10"/>
+      <c r="G62" s="26"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
         <v>306</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="D63" s="11">
-        <v>42.52</v>
+        <v>351</v>
+      </c>
+      <c r="D63" s="28">
+        <v>39.07</v>
       </c>
       <c r="E63" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="F63" s="12">
-        <v>-4.9999999997818456E-3</v>
-      </c>
-      <c r="G63" s="10"/>
+        <v>64</v>
+      </c>
+      <c r="F63" s="29">
+        <v>0</v>
+      </c>
+      <c r="G63" s="26"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
         <v>306</v>
       </c>
       <c r="B64" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D64" s="28">
+        <v>42.52</v>
+      </c>
+      <c r="E64" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="F64" s="29">
+        <v>-4.9999999997818456E-3</v>
+      </c>
+      <c r="G64" s="26"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="B65" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="C64" s="2" t="s">
+      <c r="C65" s="2" t="s">
         <v>350</v>
       </c>
-      <c r="D64" s="11">
+      <c r="D65" s="28">
         <v>39.910000000000004</v>
       </c>
-      <c r="E64" s="19" t="s">
+      <c r="E65" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="F64" s="12">
+      <c r="F65" s="29">
         <v>0</v>
       </c>
-      <c r="G64" s="10"/>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A65" s="5"/>
-      <c r="B65" s="14" t="s">
+      <c r="G65" s="26"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66" s="5"/>
+      <c r="B66" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D65" s="11">
+      <c r="D66" s="28">
         <v>33.730000000000004</v>
       </c>
-      <c r="E65" s="19" t="s">
+      <c r="E66" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="F65" s="12">
+      <c r="F66" s="29">
         <v>0</v>
       </c>
-      <c r="G65" s="10"/>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A66" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="B66" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>346</v>
-      </c>
-      <c r="D66" s="11">
-        <v>38.94</v>
-      </c>
-      <c r="E66" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="F66" s="12">
-        <v>12.200000000000017</v>
-      </c>
-      <c r="G66" s="10"/>
+      <c r="G66" s="26"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
         <v>312</v>
       </c>
       <c r="B67" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="D67" s="28">
+        <v>38.94</v>
+      </c>
+      <c r="E67" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="F67" s="29">
+        <v>9.1500000000000163</v>
+      </c>
+      <c r="G67" s="26"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="B68" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="C68" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="D67" s="11">
+      <c r="D68" s="28">
         <v>46.37</v>
       </c>
-      <c r="E67" s="19" t="s">
+      <c r="E68" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="F67" s="12">
+      <c r="F68" s="29">
         <v>0</v>
       </c>
-      <c r="G67" s="10"/>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A68" s="5"/>
-      <c r="B68" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="D68" s="11">
-        <v>59.300000000000004</v>
-      </c>
-      <c r="E68" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="F68" s="12">
-        <v>0</v>
-      </c>
-      <c r="G68" s="10"/>
+      <c r="G68" s="26"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="5"/>
       <c r="B69" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="D69" s="11">
-        <v>88.92</v>
+        <v>138</v>
+      </c>
+      <c r="D69" s="28">
+        <v>59.300000000000004</v>
       </c>
       <c r="E69" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="F69" s="12">
+        <v>70</v>
+      </c>
+      <c r="F69" s="29">
         <v>0</v>
       </c>
-      <c r="G69" s="10"/>
+      <c r="G69" s="26"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="5"/>
       <c r="B70" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="D70" s="11">
-        <v>118.54</v>
+        <v>139</v>
+      </c>
+      <c r="D70" s="28">
+        <v>88.92</v>
       </c>
       <c r="E70" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="F70" s="12">
+        <v>71</v>
+      </c>
+      <c r="F70" s="29">
         <v>0</v>
       </c>
-      <c r="G70" s="10"/>
+      <c r="G70" s="26"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="5"/>
       <c r="B71" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="D71" s="11">
-        <v>185.26</v>
+        <v>140</v>
+      </c>
+      <c r="D71" s="28">
+        <v>118.54</v>
       </c>
       <c r="E71" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="F71" s="12">
+        <v>72</v>
+      </c>
+      <c r="F71" s="29">
         <v>0</v>
       </c>
-      <c r="G71" s="10"/>
+      <c r="G71" s="26"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="5"/>
       <c r="B72" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="D72" s="11">
-        <v>169.62</v>
+        <v>141</v>
+      </c>
+      <c r="D72" s="28">
+        <v>185.26</v>
       </c>
       <c r="E72" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="F72" s="12">
+        <v>73</v>
+      </c>
+      <c r="F72" s="29">
         <v>0</v>
       </c>
-      <c r="G72" s="10"/>
+      <c r="G72" s="26"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="5"/>
-      <c r="B73" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="D73" s="11">
-        <v>0.69000000000000006</v>
-      </c>
-      <c r="E73" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="F73" s="12">
-        <v>550.80000000000132</v>
-      </c>
-      <c r="G73" s="10"/>
+      <c r="B73" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="D73" s="28">
+        <v>169.62</v>
+      </c>
+      <c r="E73" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="F73" s="29">
+        <v>0</v>
+      </c>
+      <c r="G73" s="26"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="5"/>
-      <c r="B74" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="D74" s="11">
-        <v>0.54</v>
+      <c r="B74" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="D74" s="30">
+        <v>0.69000000000000006</v>
       </c>
       <c r="E74" s="19" t="s">
-        <v>200</v>
-      </c>
-      <c r="F74" s="12">
-        <v>0</v>
-      </c>
-      <c r="G74" s="10"/>
+        <v>199</v>
+      </c>
+      <c r="F74" s="31">
+        <v>550.80000000000132</v>
+      </c>
+      <c r="G74" s="26"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" s="5"/>
       <c r="B75" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="D75" s="11">
-        <v>0.35000000000000003</v>
+        <v>144</v>
+      </c>
+      <c r="D75" s="30">
+        <v>0.54</v>
       </c>
       <c r="E75" s="19" t="s">
-        <v>201</v>
-      </c>
-      <c r="F75" s="12">
+        <v>200</v>
+      </c>
+      <c r="F75" s="31">
         <v>0</v>
       </c>
       <c r="G75" s="10"/>
@@ -3401,15 +3443,15 @@
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="5"/>
       <c r="B76" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="D76" s="11">
-        <v>0.28000000000000003</v>
+        <v>145</v>
+      </c>
+      <c r="D76" s="30">
+        <v>0.35000000000000003</v>
       </c>
       <c r="E76" s="19" t="s">
-        <v>202</v>
-      </c>
-      <c r="F76" s="12">
+        <v>201</v>
+      </c>
+      <c r="F76" s="31">
         <v>0</v>
       </c>
       <c r="G76" s="10"/>
@@ -3417,37 +3459,32 @@
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="5"/>
       <c r="B77" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="D77" s="30">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="E77" s="19" t="s">
+        <v>202</v>
+      </c>
+      <c r="F77" s="31">
+        <v>0</v>
+      </c>
+      <c r="G77" s="10"/>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A78" s="5"/>
+      <c r="B78" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="D77" s="11">
+      <c r="D78" s="30">
         <v>0.64</v>
       </c>
-      <c r="E77" s="19" t="s">
+      <c r="E78" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="F77" s="12">
-        <v>0</v>
-      </c>
-      <c r="G77" s="10"/>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A78" s="5" t="s">
-        <v>303</v>
-      </c>
-      <c r="B78" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="C78" s="17" t="s">
-        <v>354</v>
-      </c>
-      <c r="D78" s="11">
-        <v>1.33</v>
-      </c>
-      <c r="E78" s="19" t="s">
-        <v>204</v>
-      </c>
-      <c r="F78" s="12">
-        <v>16</v>
+      <c r="F78" s="31">
+        <v>-30</v>
       </c>
       <c r="G78" s="10"/>
     </row>
@@ -3456,19 +3493,19 @@
         <v>303</v>
       </c>
       <c r="B79" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>355</v>
-      </c>
-      <c r="D79" s="11">
-        <v>1.49</v>
+        <v>148</v>
+      </c>
+      <c r="C79" s="17" t="s">
+        <v>354</v>
+      </c>
+      <c r="D79" s="30">
+        <v>1.33</v>
       </c>
       <c r="E79" s="19" t="s">
-        <v>205</v>
-      </c>
-      <c r="F79" s="12">
-        <v>62</v>
+        <v>204</v>
+      </c>
+      <c r="F79" s="31">
+        <v>108</v>
       </c>
       <c r="G79" s="10"/>
     </row>
@@ -3477,19 +3514,19 @@
         <v>303</v>
       </c>
       <c r="B80" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="C80" s="17" t="s">
-        <v>358</v>
-      </c>
-      <c r="D80" s="11">
-        <v>1.6300000000000001</v>
+        <v>149</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="D80" s="30">
+        <v>1.49</v>
       </c>
       <c r="E80" s="19" t="s">
-        <v>206</v>
-      </c>
-      <c r="F80" s="12">
-        <v>239</v>
+        <v>205</v>
+      </c>
+      <c r="F80" s="31">
+        <v>251</v>
       </c>
       <c r="G80" s="10"/>
     </row>
@@ -3498,19 +3535,19 @@
         <v>303</v>
       </c>
       <c r="B81" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="C81" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="D81" s="11">
-        <v>1.82</v>
+        <v>150</v>
+      </c>
+      <c r="C81" s="17" t="s">
+        <v>358</v>
+      </c>
+      <c r="D81" s="30">
+        <v>1.6300000000000001</v>
       </c>
       <c r="E81" s="19" t="s">
-        <v>207</v>
-      </c>
-      <c r="F81" s="12">
-        <v>0</v>
+        <v>206</v>
+      </c>
+      <c r="F81" s="31">
+        <v>219</v>
       </c>
       <c r="G81" s="10"/>
     </row>
@@ -3519,19 +3556,19 @@
         <v>303</v>
       </c>
       <c r="B82" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="C82" s="17" t="s">
-        <v>362</v>
-      </c>
-      <c r="D82" s="11">
-        <v>1.96</v>
+        <v>151</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="D82" s="30">
+        <v>1.82</v>
       </c>
       <c r="E82" s="19" t="s">
-        <v>208</v>
-      </c>
-      <c r="F82" s="12">
-        <v>13</v>
+        <v>207</v>
+      </c>
+      <c r="F82" s="31">
+        <v>198</v>
       </c>
       <c r="G82" s="10"/>
     </row>
@@ -3540,19 +3577,19 @@
         <v>303</v>
       </c>
       <c r="B83" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="D83" s="11">
-        <v>2.13</v>
+        <v>152</v>
+      </c>
+      <c r="C83" s="17" t="s">
+        <v>362</v>
+      </c>
+      <c r="D83" s="30">
+        <v>1.96</v>
       </c>
       <c r="E83" s="19" t="s">
-        <v>209</v>
-      </c>
-      <c r="F83" s="12">
-        <v>125</v>
+        <v>208</v>
+      </c>
+      <c r="F83" s="31">
+        <v>213</v>
       </c>
       <c r="G83" s="10"/>
     </row>
@@ -3561,19 +3598,19 @@
         <v>303</v>
       </c>
       <c r="B84" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="C84" s="17" t="s">
-        <v>370</v>
-      </c>
-      <c r="D84" s="11">
-        <v>2.29</v>
+        <v>153</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D84" s="30">
+        <v>2.13</v>
       </c>
       <c r="E84" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="F84" s="12">
-        <v>65</v>
+        <v>209</v>
+      </c>
+      <c r="F84" s="31">
+        <v>125</v>
       </c>
       <c r="G84" s="10"/>
     </row>
@@ -3582,19 +3619,19 @@
         <v>303</v>
       </c>
       <c r="B85" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="D85" s="11">
-        <v>2.4700000000000002</v>
+        <v>154</v>
+      </c>
+      <c r="C85" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="D85" s="30">
+        <v>2.29</v>
       </c>
       <c r="E85" s="19" t="s">
-        <v>211</v>
-      </c>
-      <c r="F85" s="12">
-        <v>2</v>
+        <v>210</v>
+      </c>
+      <c r="F85" s="31">
+        <v>63</v>
       </c>
       <c r="G85" s="10"/>
     </row>
@@ -3603,19 +3640,19 @@
         <v>303</v>
       </c>
       <c r="B86" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="C86" s="17" t="s">
-        <v>371</v>
-      </c>
-      <c r="D86" s="11">
-        <v>2.61</v>
+        <v>155</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="D86" s="30">
+        <v>2.4700000000000002</v>
       </c>
       <c r="E86" s="19" t="s">
-        <v>212</v>
-      </c>
-      <c r="F86" s="12">
-        <v>0</v>
+        <v>211</v>
+      </c>
+      <c r="F86" s="31">
+        <v>2</v>
       </c>
       <c r="G86" s="10"/>
     </row>
@@ -3624,19 +3661,19 @@
         <v>303</v>
       </c>
       <c r="B87" s="13" t="s">
-        <v>459</v>
+        <v>156</v>
       </c>
       <c r="C87" s="17" t="s">
-        <v>458</v>
-      </c>
-      <c r="D87" s="11">
-        <v>1.59</v>
-      </c>
-      <c r="E87" s="10" t="s">
-        <v>457</v>
-      </c>
-      <c r="F87" s="12">
-        <v>82</v>
+        <v>371</v>
+      </c>
+      <c r="D87" s="30">
+        <v>2.61</v>
+      </c>
+      <c r="E87" s="19" t="s">
+        <v>212</v>
+      </c>
+      <c r="F87" s="31">
+        <v>0</v>
       </c>
       <c r="G87" s="10"/>
     </row>
@@ -3645,19 +3682,19 @@
         <v>303</v>
       </c>
       <c r="B88" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="C88" s="2" t="s">
-        <v>363</v>
-      </c>
-      <c r="D88" s="11">
-        <v>1.98</v>
-      </c>
-      <c r="E88" s="19" t="s">
-        <v>213</v>
-      </c>
-      <c r="F88" s="12">
-        <v>-3</v>
+        <v>459</v>
+      </c>
+      <c r="C88" s="17" t="s">
+        <v>458</v>
+      </c>
+      <c r="D88" s="30">
+        <v>1.59</v>
+      </c>
+      <c r="E88" s="10" t="s">
+        <v>457</v>
+      </c>
+      <c r="F88" s="31">
+        <v>67</v>
       </c>
       <c r="G88" s="10"/>
     </row>
@@ -3666,19 +3703,19 @@
         <v>303</v>
       </c>
       <c r="B89" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>364</v>
-      </c>
-      <c r="D89" s="11">
-        <v>2.38</v>
+        <v>363</v>
+      </c>
+      <c r="D89" s="30">
+        <v>1.98</v>
       </c>
       <c r="E89" s="19" t="s">
-        <v>214</v>
-      </c>
-      <c r="F89" s="12">
-        <v>0</v>
+        <v>213</v>
+      </c>
+      <c r="F89" s="31">
+        <v>-43</v>
       </c>
       <c r="G89" s="10"/>
     </row>
@@ -3687,56 +3724,56 @@
         <v>303</v>
       </c>
       <c r="B90" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="D90" s="30">
+        <v>2.38</v>
+      </c>
+      <c r="E90" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="F90" s="31">
+        <v>-45</v>
+      </c>
+      <c r="G90" s="10"/>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A91" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="B91" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="C90" s="2" t="s">
+      <c r="C91" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="D90" s="11">
+      <c r="D91" s="30">
         <v>2.7600000000000002</v>
       </c>
-      <c r="E90" s="19" t="s">
+      <c r="E91" s="19" t="s">
         <v>215</v>
       </c>
-      <c r="F90" s="12">
-        <v>-40</v>
-      </c>
-      <c r="G90" s="10"/>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A91" s="5"/>
-      <c r="B91" s="16" t="s">
+      <c r="F91" s="31">
+        <v>57</v>
+      </c>
+      <c r="G91" s="10"/>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A92" s="5"/>
+      <c r="B92" s="16" t="s">
         <v>160</v>
       </c>
-      <c r="D91" s="11">
+      <c r="D92" s="30">
         <v>1.31</v>
       </c>
-      <c r="E91" s="19" t="s">
+      <c r="E92" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="F91" s="12">
+      <c r="F92" s="31">
         <v>0</v>
-      </c>
-      <c r="G91" s="10"/>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A92" s="5" t="s">
-        <v>310</v>
-      </c>
-      <c r="B92" s="13" t="s">
-        <v>161</v>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="D92" s="11">
-        <v>3.12</v>
-      </c>
-      <c r="E92" s="19" t="s">
-        <v>217</v>
-      </c>
-      <c r="F92" s="12">
-        <v>-5</v>
       </c>
       <c r="G92" s="10"/>
     </row>
@@ -3745,19 +3782,19 @@
         <v>310</v>
       </c>
       <c r="B93" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="D93" s="11">
-        <v>3.5100000000000002</v>
+        <v>356</v>
+      </c>
+      <c r="D93" s="30">
+        <v>3.12</v>
       </c>
       <c r="E93" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="F93" s="12">
-        <v>34</v>
+        <v>217</v>
+      </c>
+      <c r="F93" s="31">
+        <v>13</v>
       </c>
       <c r="G93" s="10"/>
     </row>
@@ -3766,19 +3803,19 @@
         <v>310</v>
       </c>
       <c r="B94" s="13" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>359</v>
-      </c>
-      <c r="D94" s="11">
-        <v>3.91</v>
+        <v>357</v>
+      </c>
+      <c r="D94" s="30">
+        <v>3.5100000000000002</v>
       </c>
       <c r="E94" s="19" t="s">
-        <v>219</v>
-      </c>
-      <c r="F94" s="12">
-        <v>82</v>
+        <v>218</v>
+      </c>
+      <c r="F94" s="31">
+        <v>118</v>
       </c>
       <c r="G94" s="10"/>
     </row>
@@ -3787,19 +3824,19 @@
         <v>310</v>
       </c>
       <c r="B95" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>361</v>
-      </c>
-      <c r="D95" s="11">
-        <v>4.3100000000000005</v>
+        <v>359</v>
+      </c>
+      <c r="D95" s="30">
+        <v>3.91</v>
       </c>
       <c r="E95" s="19" t="s">
-        <v>220</v>
-      </c>
-      <c r="F95" s="12">
-        <v>64</v>
+        <v>219</v>
+      </c>
+      <c r="F95" s="31">
+        <v>-12</v>
       </c>
       <c r="G95" s="10"/>
     </row>
@@ -3808,19 +3845,19 @@
         <v>310</v>
       </c>
       <c r="B96" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="D96" s="11">
-        <v>4.68</v>
+        <v>361</v>
+      </c>
+      <c r="D96" s="30">
+        <v>4.3100000000000005</v>
       </c>
       <c r="E96" s="19" t="s">
-        <v>221</v>
-      </c>
-      <c r="F96" s="12">
-        <v>61</v>
+        <v>220</v>
+      </c>
+      <c r="F96" s="31">
+        <v>0</v>
       </c>
       <c r="G96" s="10"/>
     </row>
@@ -3829,19 +3866,19 @@
         <v>310</v>
       </c>
       <c r="B97" s="13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="D97" s="11">
-        <v>5.07</v>
+        <v>366</v>
+      </c>
+      <c r="D97" s="30">
+        <v>4.68</v>
       </c>
       <c r="E97" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="F97" s="12">
-        <v>66</v>
+        <v>221</v>
+      </c>
+      <c r="F97" s="31">
+        <v>48</v>
       </c>
       <c r="G97" s="10"/>
     </row>
@@ -3850,19 +3887,19 @@
         <v>310</v>
       </c>
       <c r="B98" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="D98" s="11">
-        <v>5.47</v>
+        <v>367</v>
+      </c>
+      <c r="D98" s="30">
+        <v>5.07</v>
       </c>
       <c r="E98" s="19" t="s">
-        <v>223</v>
-      </c>
-      <c r="F98" s="12">
-        <v>113</v>
+        <v>222</v>
+      </c>
+      <c r="F98" s="31">
+        <v>52</v>
       </c>
       <c r="G98" s="10"/>
     </row>
@@ -3871,56 +3908,56 @@
         <v>310</v>
       </c>
       <c r="B99" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D99" s="30">
+        <v>5.47</v>
+      </c>
+      <c r="E99" s="19" t="s">
+        <v>223</v>
+      </c>
+      <c r="F99" s="31">
+        <v>113</v>
+      </c>
+      <c r="G99" s="10"/>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A100" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="B100" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="C99" s="2" t="s">
+      <c r="C100" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="D99" s="11">
+      <c r="D100" s="30">
         <v>5.87</v>
       </c>
-      <c r="E99" s="19" t="s">
+      <c r="E100" s="19" t="s">
         <v>224</v>
       </c>
-      <c r="F99" s="12">
+      <c r="F100" s="31">
         <v>28</v>
       </c>
-      <c r="G99" s="10"/>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A100" s="5"/>
-      <c r="B100" s="16" t="s">
+      <c r="G100" s="10"/>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A101" s="5"/>
+      <c r="B101" s="16" t="s">
         <v>169</v>
       </c>
-      <c r="D100" s="11">
+      <c r="D101" s="30">
         <v>1.69</v>
       </c>
-      <c r="E100" s="19" t="s">
+      <c r="E101" s="19" t="s">
         <v>225</v>
       </c>
-      <c r="F100" s="12">
+      <c r="F101" s="31">
         <v>91</v>
-      </c>
-      <c r="G100" s="10"/>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A101" s="5" t="s">
-        <v>310</v>
-      </c>
-      <c r="B101" s="13" t="s">
-        <v>170</v>
-      </c>
-      <c r="C101" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="D101" s="11">
-        <v>3.98</v>
-      </c>
-      <c r="E101" s="19" t="s">
-        <v>226</v>
-      </c>
-      <c r="F101" s="12">
-        <v>55</v>
       </c>
       <c r="G101" s="10"/>
     </row>
@@ -3929,19 +3966,19 @@
         <v>310</v>
       </c>
       <c r="B102" s="13" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="D102" s="11">
-        <v>5.12</v>
+        <v>372</v>
+      </c>
+      <c r="D102" s="30">
+        <v>4.0999999999999996</v>
       </c>
       <c r="E102" s="19" t="s">
-        <v>227</v>
-      </c>
-      <c r="F102" s="12">
-        <v>45</v>
+        <v>226</v>
+      </c>
+      <c r="F102" s="31">
+        <v>105</v>
       </c>
       <c r="G102" s="10"/>
     </row>
@@ -3950,19 +3987,19 @@
         <v>310</v>
       </c>
       <c r="B103" s="13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>375</v>
-      </c>
-      <c r="D103" s="11">
-        <v>5.94</v>
+        <v>374</v>
+      </c>
+      <c r="D103" s="30">
+        <v>5.12</v>
       </c>
       <c r="E103" s="19" t="s">
-        <v>228</v>
-      </c>
-      <c r="F103" s="12">
-        <v>52</v>
+        <v>227</v>
+      </c>
+      <c r="F103" s="31">
+        <v>86</v>
       </c>
       <c r="G103" s="10"/>
     </row>
@@ -3971,56 +4008,56 @@
         <v>310</v>
       </c>
       <c r="B104" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="D104" s="30">
+        <v>6.13</v>
+      </c>
+      <c r="E104" s="19" t="s">
+        <v>228</v>
+      </c>
+      <c r="F104" s="31">
+        <v>49</v>
+      </c>
+      <c r="G104" s="10"/>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A105" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="B105" s="13" t="s">
         <v>173</v>
       </c>
-      <c r="C104" s="2" t="s">
+      <c r="C105" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="D104" s="11">
-        <v>6.92</v>
-      </c>
-      <c r="E104" s="19" t="s">
+      <c r="D105" s="30">
+        <v>7.15</v>
+      </c>
+      <c r="E105" s="19" t="s">
         <v>229</v>
       </c>
-      <c r="F104" s="12">
-        <v>41</v>
-      </c>
-      <c r="G104" s="10"/>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A105" s="5"/>
-      <c r="B105" s="16" t="s">
+      <c r="F105" s="31">
+        <v>33</v>
+      </c>
+      <c r="G105" s="10"/>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A106" s="5"/>
+      <c r="B106" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="D105" s="11">
+      <c r="D106" s="30">
         <v>2.13</v>
       </c>
-      <c r="E105" s="19" t="s">
+      <c r="E106" s="19" t="s">
         <v>230</v>
       </c>
-      <c r="F105" s="12">
+      <c r="F106" s="31">
         <v>0</v>
-      </c>
-      <c r="G105" s="10"/>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A106" s="5" t="s">
-        <v>302</v>
-      </c>
-      <c r="B106" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="C106" s="2" t="s">
-        <v>373</v>
-      </c>
-      <c r="D106" s="11">
-        <v>5.1100000000000003</v>
-      </c>
-      <c r="E106" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="F106" s="12">
-        <v>-7</v>
       </c>
       <c r="G106" s="10"/>
     </row>
@@ -4029,19 +4066,19 @@
         <v>302</v>
       </c>
       <c r="B107" s="13" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="D107" s="11">
-        <v>5.76</v>
+        <v>373</v>
+      </c>
+      <c r="D107" s="30">
+        <v>5.1100000000000003</v>
       </c>
       <c r="E107" s="19" t="s">
-        <v>232</v>
-      </c>
-      <c r="F107" s="12">
-        <v>100</v>
+        <v>231</v>
+      </c>
+      <c r="F107" s="31">
+        <v>21</v>
       </c>
       <c r="G107" s="10"/>
     </row>
@@ -4050,19 +4087,19 @@
         <v>302</v>
       </c>
       <c r="B108" s="13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>389</v>
-      </c>
-      <c r="D108" s="11">
-        <v>6.3900000000000006</v>
+        <v>379</v>
+      </c>
+      <c r="D108" s="30">
+        <v>5.76</v>
       </c>
       <c r="E108" s="19" t="s">
-        <v>233</v>
-      </c>
-      <c r="F108" s="12">
-        <v>13</v>
+        <v>232</v>
+      </c>
+      <c r="F108" s="31">
+        <v>95</v>
       </c>
       <c r="G108" s="10"/>
     </row>
@@ -4071,19 +4108,19 @@
         <v>302</v>
       </c>
       <c r="B109" s="13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="D109" s="11">
-        <v>7.03</v>
+        <v>389</v>
+      </c>
+      <c r="D109" s="30">
+        <v>6.3900000000000006</v>
       </c>
       <c r="E109" s="19" t="s">
-        <v>234</v>
-      </c>
-      <c r="F109" s="12">
-        <v>31</v>
+        <v>233</v>
+      </c>
+      <c r="F109" s="31">
+        <v>93</v>
       </c>
       <c r="G109" s="10"/>
     </row>
@@ -4092,19 +4129,19 @@
         <v>302</v>
       </c>
       <c r="B110" s="13" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="D110" s="11">
-        <v>7.68</v>
+        <v>390</v>
+      </c>
+      <c r="D110" s="30">
+        <v>7.03</v>
       </c>
       <c r="E110" s="19" t="s">
-        <v>235</v>
-      </c>
-      <c r="F110" s="12">
-        <v>95</v>
+        <v>234</v>
+      </c>
+      <c r="F110" s="31">
+        <v>31</v>
       </c>
       <c r="G110" s="10"/>
     </row>
@@ -4113,19 +4150,19 @@
         <v>302</v>
       </c>
       <c r="B111" s="13" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="D111" s="11">
-        <v>8.31</v>
+        <v>391</v>
+      </c>
+      <c r="D111" s="30">
+        <v>7.68</v>
       </c>
       <c r="E111" s="19" t="s">
-        <v>236</v>
-      </c>
-      <c r="F111" s="12">
-        <v>148</v>
+        <v>235</v>
+      </c>
+      <c r="F111" s="31">
+        <v>83</v>
       </c>
       <c r="G111" s="10"/>
     </row>
@@ -4134,19 +4171,19 @@
         <v>302</v>
       </c>
       <c r="B112" s="13" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="D112" s="11">
-        <v>8.9500000000000011</v>
+        <v>392</v>
+      </c>
+      <c r="D112" s="30">
+        <v>8.31</v>
       </c>
       <c r="E112" s="19" t="s">
-        <v>237</v>
-      </c>
-      <c r="F112" s="12">
-        <v>4</v>
+        <v>236</v>
+      </c>
+      <c r="F112" s="31">
+        <v>144</v>
       </c>
       <c r="G112" s="10"/>
     </row>
@@ -4155,56 +4192,56 @@
         <v>302</v>
       </c>
       <c r="B113" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="D113" s="30">
+        <v>8.9500000000000011</v>
+      </c>
+      <c r="E113" s="19" t="s">
+        <v>237</v>
+      </c>
+      <c r="F113" s="31">
+        <v>16</v>
+      </c>
+      <c r="G113" s="10"/>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A114" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="B114" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="C113" s="2" t="s">
+      <c r="C114" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="D113" s="11">
+      <c r="D114" s="30">
         <v>9.61</v>
       </c>
-      <c r="E113" s="19" t="s">
+      <c r="E114" s="19" t="s">
         <v>238</v>
       </c>
-      <c r="F113" s="12">
+      <c r="F114" s="31">
         <v>8</v>
       </c>
-      <c r="G113" s="10"/>
-    </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A114" s="5"/>
-      <c r="B114" s="16" t="s">
+      <c r="G114" s="10"/>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A115" s="5"/>
+      <c r="B115" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="D114" s="11">
+      <c r="D115" s="30">
         <v>4.2700000000000005</v>
       </c>
-      <c r="E114" s="19" t="s">
+      <c r="E115" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="F114" s="12">
+      <c r="F115" s="31">
         <v>0</v>
-      </c>
-      <c r="G114" s="10"/>
-    </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A115" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="B115" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="C115" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="D115" s="11">
-        <v>10.220000000000001</v>
-      </c>
-      <c r="E115" s="19" t="s">
-        <v>240</v>
-      </c>
-      <c r="F115" s="12">
-        <v>20</v>
       </c>
       <c r="G115" s="10"/>
     </row>
@@ -4213,19 +4250,19 @@
         <v>308</v>
       </c>
       <c r="B116" s="13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="D116" s="11">
-        <v>11.5</v>
+        <v>380</v>
+      </c>
+      <c r="D116" s="30">
+        <v>10.220000000000001</v>
       </c>
       <c r="E116" s="19" t="s">
-        <v>241</v>
-      </c>
-      <c r="F116" s="12">
-        <v>14</v>
+        <v>240</v>
+      </c>
+      <c r="F116" s="31">
+        <v>17</v>
       </c>
       <c r="G116" s="10"/>
     </row>
@@ -4234,19 +4271,19 @@
         <v>308</v>
       </c>
       <c r="B117" s="13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>382</v>
-      </c>
-      <c r="D117" s="11">
-        <v>12.780000000000001</v>
+        <v>381</v>
+      </c>
+      <c r="D117" s="30">
+        <v>11.5</v>
       </c>
       <c r="E117" s="19" t="s">
-        <v>242</v>
-      </c>
-      <c r="F117" s="12">
-        <v>8</v>
+        <v>241</v>
+      </c>
+      <c r="F117" s="31">
+        <v>20</v>
       </c>
       <c r="G117" s="10"/>
     </row>
@@ -4255,19 +4292,19 @@
         <v>308</v>
       </c>
       <c r="B118" s="13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="D118" s="11">
-        <v>14.07</v>
+        <v>382</v>
+      </c>
+      <c r="D118" s="30">
+        <v>12.780000000000001</v>
       </c>
       <c r="E118" s="19" t="s">
-        <v>243</v>
-      </c>
-      <c r="F118" s="12">
-        <v>12</v>
+        <v>242</v>
+      </c>
+      <c r="F118" s="31">
+        <v>20</v>
       </c>
       <c r="G118" s="10"/>
     </row>
@@ -4276,19 +4313,19 @@
         <v>308</v>
       </c>
       <c r="B119" s="13" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="D119" s="11">
-        <v>15.34</v>
+        <v>383</v>
+      </c>
+      <c r="D119" s="30">
+        <v>14.07</v>
       </c>
       <c r="E119" s="19" t="s">
-        <v>244</v>
-      </c>
-      <c r="F119" s="12">
-        <v>15</v>
+        <v>243</v>
+      </c>
+      <c r="F119" s="31">
+        <v>19</v>
       </c>
       <c r="G119" s="10"/>
     </row>
@@ -4297,19 +4334,19 @@
         <v>308</v>
       </c>
       <c r="B120" s="13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>385</v>
-      </c>
-      <c r="D120" s="11">
-        <v>16.61</v>
+        <v>384</v>
+      </c>
+      <c r="D120" s="30">
+        <v>15.34</v>
       </c>
       <c r="E120" s="19" t="s">
-        <v>245</v>
-      </c>
-      <c r="F120" s="12">
-        <v>32</v>
+        <v>244</v>
+      </c>
+      <c r="F120" s="31">
+        <v>20</v>
       </c>
       <c r="G120" s="10"/>
     </row>
@@ -4318,19 +4355,19 @@
         <v>308</v>
       </c>
       <c r="B121" s="13" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>386</v>
-      </c>
-      <c r="D121" s="11">
-        <v>17.88</v>
+        <v>385</v>
+      </c>
+      <c r="D121" s="30">
+        <v>16.61</v>
       </c>
       <c r="E121" s="19" t="s">
-        <v>246</v>
-      </c>
-      <c r="F121" s="12">
-        <v>21</v>
+        <v>245</v>
+      </c>
+      <c r="F121" s="31">
+        <v>38</v>
       </c>
       <c r="G121" s="10"/>
     </row>
@@ -4339,56 +4376,56 @@
         <v>308</v>
       </c>
       <c r="B122" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="D122" s="30">
+        <v>17.88</v>
+      </c>
+      <c r="E122" s="19" t="s">
+        <v>246</v>
+      </c>
+      <c r="F122" s="31">
+        <v>21</v>
+      </c>
+      <c r="G122" s="10"/>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A123" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="B123" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="C122" s="2" t="s">
+      <c r="C123" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="D122" s="11">
+      <c r="D123" s="30">
         <v>19.12</v>
       </c>
-      <c r="E122" s="19" t="s">
+      <c r="E123" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="F122" s="12">
+      <c r="F123" s="31">
         <v>11</v>
       </c>
-      <c r="G122" s="10"/>
-    </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A123" s="5"/>
-      <c r="B123" s="16" t="s">
+      <c r="G123" s="10"/>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A124" s="5"/>
+      <c r="B124" s="16" t="s">
         <v>192</v>
       </c>
-      <c r="D123" s="11">
+      <c r="D124" s="30">
         <v>8.02</v>
       </c>
-      <c r="E123" s="19" t="s">
+      <c r="E124" s="19" t="s">
         <v>248</v>
       </c>
-      <c r="F123" s="12">
+      <c r="F124" s="31">
         <v>0</v>
-      </c>
-      <c r="G123" s="10"/>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A124" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="B124" s="13" t="s">
-        <v>193</v>
-      </c>
-      <c r="C124" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="D124" s="11">
-        <v>18.100000000000001</v>
-      </c>
-      <c r="E124" s="19" t="s">
-        <v>249</v>
-      </c>
-      <c r="F124" s="12">
-        <v>13</v>
       </c>
       <c r="G124" s="10"/>
     </row>
@@ -4397,19 +4434,19 @@
         <v>308</v>
       </c>
       <c r="B125" s="13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="D125" s="11">
-        <v>22.64</v>
+        <v>388</v>
+      </c>
+      <c r="D125" s="30">
+        <v>18.100000000000001</v>
       </c>
       <c r="E125" s="19" t="s">
-        <v>250</v>
-      </c>
-      <c r="F125" s="12">
-        <v>16</v>
+        <v>249</v>
+      </c>
+      <c r="F125" s="31">
+        <v>13</v>
       </c>
       <c r="G125" s="10"/>
     </row>
@@ -4418,19 +4455,19 @@
         <v>308</v>
       </c>
       <c r="B126" s="13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="D126" s="11">
-        <v>27.150000000000002</v>
+        <v>395</v>
+      </c>
+      <c r="D126" s="30">
+        <v>22.64</v>
       </c>
       <c r="E126" s="19" t="s">
-        <v>251</v>
-      </c>
-      <c r="F126" s="12">
-        <v>21</v>
+        <v>250</v>
+      </c>
+      <c r="F126" s="31">
+        <v>5</v>
       </c>
       <c r="G126" s="10"/>
     </row>
@@ -4439,19 +4476,19 @@
         <v>308</v>
       </c>
       <c r="B127" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="D127" s="11">
-        <v>31.69</v>
+        <v>396</v>
+      </c>
+      <c r="D127" s="30">
+        <v>27.150000000000002</v>
       </c>
       <c r="E127" s="19" t="s">
-        <v>252</v>
-      </c>
-      <c r="F127" s="12">
-        <v>15</v>
+        <v>251</v>
+      </c>
+      <c r="F127" s="31">
+        <v>21</v>
       </c>
       <c r="G127" s="10"/>
     </row>
@@ -4460,19 +4497,19 @@
         <v>308</v>
       </c>
       <c r="B128" s="13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="D128" s="11">
-        <v>33.94</v>
+        <v>397</v>
+      </c>
+      <c r="D128" s="30">
+        <v>31.69</v>
       </c>
       <c r="E128" s="19" t="s">
-        <v>253</v>
-      </c>
-      <c r="F128" s="12">
-        <v>0</v>
+        <v>252</v>
+      </c>
+      <c r="F128" s="31">
+        <v>14</v>
       </c>
       <c r="G128" s="10"/>
     </row>
@@ -4481,55 +4518,55 @@
         <v>308</v>
       </c>
       <c r="B129" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="D129" s="30">
+        <v>33.94</v>
+      </c>
+      <c r="E129" s="19" t="s">
+        <v>253</v>
+      </c>
+      <c r="F129" s="31">
+        <v>0</v>
+      </c>
+      <c r="G129" s="10"/>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A130" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="B130" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="C129" s="2" t="s">
+      <c r="C130" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="D129" s="11">
+      <c r="D130" s="30">
         <v>36.22</v>
       </c>
-      <c r="E129" s="19" t="s">
+      <c r="E130" s="19" t="s">
         <v>254</v>
       </c>
-      <c r="F129" s="12">
+      <c r="F130" s="31">
         <v>0</v>
       </c>
-      <c r="G129" s="10"/>
-    </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A130" s="5"/>
-      <c r="B130" s="15" t="s">
+      <c r="G130" s="10"/>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A131" s="5"/>
+      <c r="B131" s="15" t="s">
         <v>278</v>
       </c>
-      <c r="D130" s="11">
+      <c r="D131" s="32">
         <v>2.15</v>
       </c>
-      <c r="E130" s="19" t="s">
+      <c r="E131" s="19" t="s">
         <v>255</v>
       </c>
-      <c r="F130" s="12">
-        <v>0</v>
-      </c>
-      <c r="G130" s="10"/>
-    </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A131" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="B131" s="10" t="s">
-        <v>279</v>
-      </c>
-      <c r="C131" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="D131" s="11">
-        <v>5.12</v>
-      </c>
-      <c r="E131" s="19" t="s">
-        <v>256</v>
-      </c>
-      <c r="F131" s="12">
+      <c r="F131" s="33">
         <v>0</v>
       </c>
       <c r="G131" s="10"/>
@@ -4539,19 +4576,19 @@
         <v>309</v>
       </c>
       <c r="B132" s="10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>401</v>
-      </c>
-      <c r="D132" s="11">
-        <v>3.93</v>
+        <v>400</v>
+      </c>
+      <c r="D132" s="32">
+        <v>5.12</v>
       </c>
       <c r="E132" s="19" t="s">
-        <v>257</v>
-      </c>
-      <c r="F132" s="12">
-        <v>369</v>
+        <v>256</v>
+      </c>
+      <c r="F132" s="33">
+        <v>0</v>
       </c>
       <c r="G132" s="10"/>
     </row>
@@ -4560,19 +4597,19 @@
         <v>309</v>
       </c>
       <c r="B133" s="10" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>402</v>
-      </c>
-      <c r="D133" s="11">
-        <v>4.53</v>
+        <v>401</v>
+      </c>
+      <c r="D133" s="32">
+        <v>3.93</v>
       </c>
       <c r="E133" s="19" t="s">
-        <v>258</v>
-      </c>
-      <c r="F133" s="12">
-        <v>624</v>
+        <v>257</v>
+      </c>
+      <c r="F133" s="33">
+        <v>-99</v>
       </c>
       <c r="G133" s="10"/>
     </row>
@@ -4581,19 +4618,19 @@
         <v>309</v>
       </c>
       <c r="B134" s="10" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>403</v>
-      </c>
-      <c r="D134" s="11">
-        <v>6.7</v>
+        <v>402</v>
+      </c>
+      <c r="D134" s="32">
+        <v>4.53</v>
       </c>
       <c r="E134" s="19" t="s">
-        <v>259</v>
-      </c>
-      <c r="F134" s="12">
-        <v>193</v>
+        <v>258</v>
+      </c>
+      <c r="F134" s="33">
+        <v>396</v>
       </c>
       <c r="G134" s="10"/>
     </row>
@@ -4602,19 +4639,19 @@
         <v>309</v>
       </c>
       <c r="B135" s="10" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>404</v>
-      </c>
-      <c r="D135" s="11">
-        <v>8.31</v>
+        <v>403</v>
+      </c>
+      <c r="D135" s="32">
+        <v>6.7</v>
       </c>
       <c r="E135" s="19" t="s">
-        <v>260</v>
-      </c>
-      <c r="F135" s="12">
-        <v>0</v>
+        <v>259</v>
+      </c>
+      <c r="F135" s="33">
+        <v>193</v>
       </c>
       <c r="G135" s="10"/>
     </row>
@@ -4623,19 +4660,19 @@
         <v>309</v>
       </c>
       <c r="B136" s="10" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>405</v>
-      </c>
-      <c r="D136" s="11">
-        <v>7.8900000000000006</v>
+        <v>404</v>
+      </c>
+      <c r="D136" s="32">
+        <v>8.31</v>
       </c>
       <c r="E136" s="19" t="s">
-        <v>261</v>
-      </c>
-      <c r="F136" s="12">
-        <v>369</v>
+        <v>260</v>
+      </c>
+      <c r="F136" s="33">
+        <v>0</v>
       </c>
       <c r="G136" s="10"/>
     </row>
@@ -4644,56 +4681,56 @@
         <v>309</v>
       </c>
       <c r="B137" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="D137" s="32">
+        <v>7.8900000000000006</v>
+      </c>
+      <c r="E137" s="19" t="s">
+        <v>261</v>
+      </c>
+      <c r="F137" s="33">
+        <v>357</v>
+      </c>
+      <c r="G137" s="10"/>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A138" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="B138" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="C137" s="2" t="s">
+      <c r="C138" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="D137" s="11">
+      <c r="D138" s="32">
         <v>9.61</v>
       </c>
-      <c r="E137" s="19" t="s">
+      <c r="E138" s="19" t="s">
         <v>262</v>
       </c>
-      <c r="F137" s="12">
+      <c r="F138" s="33">
         <v>0</v>
       </c>
-      <c r="G137" s="10"/>
-    </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A138" s="5"/>
-      <c r="B138" s="15" t="s">
+      <c r="G138" s="10"/>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A139" s="5"/>
+      <c r="B139" s="15" t="s">
         <v>286</v>
       </c>
-      <c r="D138" s="11">
+      <c r="D139" s="32">
         <v>3.5500000000000003</v>
       </c>
-      <c r="E138" s="19" t="s">
+      <c r="E139" s="19" t="s">
         <v>263</v>
       </c>
-      <c r="F138" s="12">
+      <c r="F139" s="33">
         <v>0</v>
-      </c>
-      <c r="G138" s="10"/>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A139" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="B139" s="10" t="s">
-        <v>287</v>
-      </c>
-      <c r="C139" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="D139" s="11">
-        <v>6.22</v>
-      </c>
-      <c r="E139" s="19" t="s">
-        <v>264</v>
-      </c>
-      <c r="F139" s="12">
-        <v>239</v>
       </c>
       <c r="G139" s="10"/>
     </row>
@@ -4702,19 +4739,19 @@
         <v>309</v>
       </c>
       <c r="B140" s="10" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="D140" s="11">
-        <v>6.7</v>
+        <v>407</v>
+      </c>
+      <c r="D140" s="32">
+        <v>6.22</v>
       </c>
       <c r="E140" s="19" t="s">
-        <v>265</v>
-      </c>
-      <c r="F140" s="12">
-        <v>375</v>
+        <v>264</v>
+      </c>
+      <c r="F140" s="33">
+        <v>221</v>
       </c>
       <c r="G140" s="10"/>
     </row>
@@ -4723,19 +4760,19 @@
         <v>309</v>
       </c>
       <c r="B141" s="10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="D141" s="11">
-        <v>10.91</v>
+        <v>414</v>
+      </c>
+      <c r="D141" s="32">
+        <v>6.7</v>
       </c>
       <c r="E141" s="19" t="s">
-        <v>266</v>
-      </c>
-      <c r="F141" s="12">
-        <v>0</v>
+        <v>265</v>
+      </c>
+      <c r="F141" s="33">
+        <v>317</v>
       </c>
       <c r="G141" s="10"/>
     </row>
@@ -4744,19 +4781,19 @@
         <v>309</v>
       </c>
       <c r="B142" s="10" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>416</v>
-      </c>
-      <c r="D142" s="11">
-        <v>10.370000000000001</v>
+        <v>415</v>
+      </c>
+      <c r="D142" s="32">
+        <v>10.91</v>
       </c>
       <c r="E142" s="19" t="s">
-        <v>267</v>
-      </c>
-      <c r="F142" s="12">
-        <v>201</v>
+        <v>266</v>
+      </c>
+      <c r="F142" s="33">
+        <v>0</v>
       </c>
       <c r="G142" s="10"/>
     </row>
@@ -4765,19 +4802,19 @@
         <v>309</v>
       </c>
       <c r="B143" s="10" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>417</v>
-      </c>
-      <c r="D143" s="11">
-        <v>6.76</v>
+        <v>416</v>
+      </c>
+      <c r="D143" s="32">
+        <v>10.370000000000001</v>
       </c>
       <c r="E143" s="19" t="s">
-        <v>268</v>
-      </c>
-      <c r="F143" s="12">
-        <v>132</v>
+        <v>267</v>
+      </c>
+      <c r="F143" s="33">
+        <v>194</v>
       </c>
       <c r="G143" s="10"/>
     </row>
@@ -4786,19 +4823,19 @@
         <v>309</v>
       </c>
       <c r="B144" s="10" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>418</v>
-      </c>
-      <c r="D144" s="11">
-        <v>9.23</v>
+        <v>417</v>
+      </c>
+      <c r="D144" s="32">
+        <v>6.76</v>
       </c>
       <c r="E144" s="19" t="s">
-        <v>269</v>
-      </c>
-      <c r="F144" s="12">
-        <v>0</v>
+        <v>268</v>
+      </c>
+      <c r="F144" s="33">
+        <v>126</v>
       </c>
       <c r="G144" s="10"/>
     </row>
@@ -4807,55 +4844,55 @@
         <v>309</v>
       </c>
       <c r="B145" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="D145" s="32">
+        <v>9.23</v>
+      </c>
+      <c r="E145" s="19" t="s">
+        <v>269</v>
+      </c>
+      <c r="F145" s="33">
+        <v>0</v>
+      </c>
+      <c r="G145" s="10"/>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A146" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="B146" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="C145" s="2" t="s">
+      <c r="C146" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="D145" s="11">
+      <c r="D146" s="32">
         <v>11.14</v>
       </c>
-      <c r="E145" s="19" t="s">
+      <c r="E146" s="19" t="s">
         <v>270</v>
       </c>
-      <c r="F145" s="12">
+      <c r="F146" s="33">
         <v>0</v>
       </c>
-      <c r="G145" s="10"/>
-    </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A146" s="5"/>
-      <c r="B146" s="15" t="s">
+      <c r="G146" s="10"/>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A147" s="5"/>
+      <c r="B147" s="15" t="s">
         <v>294</v>
       </c>
-      <c r="D146" s="11">
+      <c r="D147" s="32">
         <v>3.17</v>
       </c>
-      <c r="E146" s="19" t="s">
+      <c r="E147" s="19" t="s">
         <v>271</v>
       </c>
-      <c r="F146" s="12">
-        <v>0</v>
-      </c>
-      <c r="G146" s="10"/>
-    </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A147" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="B147" s="10" t="s">
-        <v>295</v>
-      </c>
-      <c r="C147" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="D147" s="11">
-        <v>7.2</v>
-      </c>
-      <c r="E147" s="19" t="s">
-        <v>272</v>
-      </c>
-      <c r="F147" s="12">
+      <c r="F147" s="33">
         <v>0</v>
       </c>
       <c r="G147" s="10"/>
@@ -4865,18 +4902,18 @@
         <v>309</v>
       </c>
       <c r="B148" s="10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="D148" s="11">
-        <v>18.11</v>
+        <v>408</v>
+      </c>
+      <c r="D148" s="32">
+        <v>7.2</v>
       </c>
       <c r="E148" s="19" t="s">
-        <v>273</v>
-      </c>
-      <c r="F148" s="12">
+        <v>272</v>
+      </c>
+      <c r="F148" s="33">
         <v>0</v>
       </c>
       <c r="G148" s="10"/>
@@ -4886,19 +4923,19 @@
         <v>309</v>
       </c>
       <c r="B149" s="10" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>410</v>
-      </c>
-      <c r="D149" s="11">
-        <v>11.94</v>
+        <v>409</v>
+      </c>
+      <c r="D149" s="32">
+        <v>18.11</v>
       </c>
       <c r="E149" s="19" t="s">
-        <v>274</v>
-      </c>
-      <c r="F149" s="12">
-        <v>81</v>
+        <v>273</v>
+      </c>
+      <c r="F149" s="33">
+        <v>0</v>
       </c>
       <c r="G149" s="10"/>
     </row>
@@ -4907,19 +4944,19 @@
         <v>309</v>
       </c>
       <c r="B150" s="10" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="D150" s="11">
-        <v>15.16</v>
+        <v>410</v>
+      </c>
+      <c r="D150" s="32">
+        <v>11.94</v>
       </c>
       <c r="E150" s="19" t="s">
-        <v>275</v>
-      </c>
-      <c r="F150" s="12">
-        <v>45</v>
+        <v>274</v>
+      </c>
+      <c r="F150" s="33">
+        <v>61</v>
       </c>
       <c r="G150" s="10"/>
     </row>
@@ -4928,19 +4965,19 @@
         <v>309</v>
       </c>
       <c r="B151" s="10" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="D151" s="11">
-        <v>13.52</v>
+        <v>411</v>
+      </c>
+      <c r="D151" s="32">
+        <v>15.16</v>
       </c>
       <c r="E151" s="19" t="s">
-        <v>276</v>
-      </c>
-      <c r="F151" s="12">
-        <v>43</v>
+        <v>275</v>
+      </c>
+      <c r="F151" s="33">
+        <v>45</v>
       </c>
       <c r="G151" s="10"/>
     </row>
@@ -4949,128 +4986,129 @@
         <v>309</v>
       </c>
       <c r="B152" s="10" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>413</v>
-      </c>
-      <c r="D152" s="11">
-        <v>24.89</v>
+        <v>412</v>
+      </c>
+      <c r="D152" s="32">
+        <v>13.52</v>
       </c>
       <c r="E152" s="19" t="s">
-        <v>277</v>
-      </c>
-      <c r="F152" s="12">
-        <v>0</v>
+        <v>276</v>
+      </c>
+      <c r="F152" s="33">
+        <v>43</v>
       </c>
       <c r="G152" s="10"/>
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A153" s="5" t="s">
-        <v>441</v>
-      </c>
-      <c r="B153" s="23" t="s">
-        <v>420</v>
-      </c>
-      <c r="C153" s="5" t="s">
-        <v>451</v>
-      </c>
-      <c r="D153" s="12">
-        <v>7.8</v>
+        <v>309</v>
+      </c>
+      <c r="B153" s="10" t="s">
+        <v>300</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="D153" s="32">
+        <v>24.89</v>
       </c>
       <c r="E153" s="19" t="s">
-        <v>460</v>
-      </c>
-      <c r="F153" s="22">
-        <v>2</v>
-      </c>
+        <v>277</v>
+      </c>
+      <c r="F153" s="12">
+        <v>0</v>
+      </c>
+      <c r="G153" s="10"/>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A154" s="5" t="s">
-        <v>442</v>
-      </c>
-      <c r="B154" s="24" t="s">
-        <v>421</v>
-      </c>
-      <c r="C154" s="2" t="s">
-        <v>452</v>
-      </c>
-      <c r="D154" s="11">
-        <v>18.150000000000002</v>
-      </c>
-      <c r="E154" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="F154" s="12">
-        <v>3</v>
+        <v>441</v>
+      </c>
+      <c r="B154" s="23" t="s">
+        <v>420</v>
+      </c>
+      <c r="C154" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="D154" s="12">
+        <v>7.8</v>
+      </c>
+      <c r="E154" s="19" t="s">
+        <v>460</v>
+      </c>
+      <c r="F154" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A155" s="5" t="s">
-        <v>443</v>
-      </c>
-      <c r="B155" s="13" t="s">
-        <v>424</v>
-      </c>
-      <c r="C155" s="5" t="s">
-        <v>455</v>
+        <v>442</v>
+      </c>
+      <c r="B155" s="24" t="s">
+        <v>421</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>452</v>
       </c>
       <c r="D155" s="11">
-        <v>23.8</v>
-      </c>
-      <c r="E155" s="19" t="s">
-        <v>423</v>
+        <v>18.150000000000002</v>
+      </c>
+      <c r="E155" s="10" t="s">
+        <v>422</v>
       </c>
       <c r="F155" s="12">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A156" s="5" t="s">
-        <v>444</v>
-      </c>
-      <c r="B156" s="24" t="s">
-        <v>426</v>
+        <v>443</v>
+      </c>
+      <c r="B156" s="13" t="s">
+        <v>424</v>
       </c>
       <c r="C156" s="5" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="D156" s="11">
-        <v>18.22</v>
+        <v>23.8</v>
       </c>
       <c r="E156" s="19" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="F156" s="12">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A157" s="5" t="s">
-        <v>445</v>
-      </c>
-      <c r="B157" s="9" t="s">
-        <v>427</v>
+        <v>444</v>
+      </c>
+      <c r="B157" s="24" t="s">
+        <v>426</v>
       </c>
       <c r="C157" s="5" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="D157" s="11">
-        <v>9.82</v>
-      </c>
-      <c r="E157" s="10" t="s">
-        <v>434</v>
+        <v>18.22</v>
+      </c>
+      <c r="E157" s="19" t="s">
+        <v>425</v>
       </c>
       <c r="F157" s="12">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A158" s="5" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="B158" s="9" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C158" s="5" t="s">
         <v>456</v>
@@ -5079,18 +5117,18 @@
         <v>9.82</v>
       </c>
       <c r="E158" s="10" t="s">
-        <v>435</v>
-      </c>
-      <c r="F158" s="12">
-        <v>-2</v>
+        <v>434</v>
+      </c>
+      <c r="F158" s="34">
+        <v>-1</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A159" s="5" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B159" s="9" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C159" s="5" t="s">
         <v>456</v>
@@ -5099,18 +5137,18 @@
         <v>9.82</v>
       </c>
       <c r="E159" s="10" t="s">
-        <v>436</v>
-      </c>
-      <c r="F159" s="12">
-        <v>0</v>
+        <v>435</v>
+      </c>
+      <c r="F159" s="34">
+        <v>-4</v>
       </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A160" s="5" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="B160" s="9" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C160" s="5" t="s">
         <v>456</v>
@@ -5119,18 +5157,18 @@
         <v>9.82</v>
       </c>
       <c r="E160" s="10" t="s">
-        <v>437</v>
-      </c>
-      <c r="F160" s="12">
-        <v>2</v>
+        <v>436</v>
+      </c>
+      <c r="F160" s="34">
+        <v>0</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" s="5" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="B161" s="9" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C161" s="5" t="s">
         <v>456</v>
@@ -5139,18 +5177,18 @@
         <v>9.82</v>
       </c>
       <c r="E161" s="10" t="s">
-        <v>438</v>
-      </c>
-      <c r="F161" s="12">
-        <v>0</v>
+        <v>437</v>
+      </c>
+      <c r="F161" s="34">
+        <v>1</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="5" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B162" s="9" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C162" s="5" t="s">
         <v>456</v>
@@ -5159,39 +5197,51 @@
         <v>9.82</v>
       </c>
       <c r="E162" s="10" t="s">
-        <v>439</v>
-      </c>
-      <c r="F162" s="12">
-        <v>0</v>
+        <v>438</v>
+      </c>
+      <c r="F162" s="34">
+        <v>-1</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="B163" s="9" t="s">
+        <v>432</v>
+      </c>
+      <c r="C163" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="D163" s="11">
+        <v>9.82</v>
+      </c>
+      <c r="E163" s="10" t="s">
+        <v>439</v>
+      </c>
+      <c r="F163" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A164" s="5" t="s">
         <v>446</v>
       </c>
-      <c r="B163" s="9" t="s">
+      <c r="B164" s="9" t="s">
         <v>433</v>
       </c>
-      <c r="C163" s="5" t="s">
+      <c r="C164" s="5" t="s">
         <v>454</v>
       </c>
-      <c r="D163" s="11">
+      <c r="D164" s="11">
         <v>6.3</v>
       </c>
-      <c r="E163" s="10" t="s">
+      <c r="E164" s="10" t="s">
         <v>440</v>
       </c>
-      <c r="F163" s="12">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A164" s="5"/>
-      <c r="B164" s="5"/>
-      <c r="C164" s="5"/>
-      <c r="D164" s="5"/>
-      <c r="E164" s="19"/>
-      <c r="F164" s="5"/>
+      <c r="F164" s="34">
+        <v>1</v>
+      </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" s="5"/>
@@ -7482,13 +7532,21 @@
       <c r="F450" s="5"/>
     </row>
     <row r="451" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A451" s="2"/>
+      <c r="A451" s="5"/>
+      <c r="B451" s="5"/>
+      <c r="C451" s="5"/>
+      <c r="D451" s="5"/>
+      <c r="E451" s="19"/>
+      <c r="F451" s="5"/>
     </row>
     <row r="452" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A452" s="2"/>
     </row>
     <row r="453" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A453" s="2"/>
+    </row>
+    <row r="454" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A454" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>